<commit_message>
feat(liraa): atualiza base do XLSForm e compatibiliza grupo de tratamento
Substitui app_core/data/liraa_kobo_base.xlsx pelo modelo enviado pelo
usuario (C:\LIRAa.xlsx). Ajustes de compatibilidade:

- grupo de tratamento renomeado group_rb5ho54 -> tratamento_001;
- campo 'foi tratado' renomeado O_im_vel_foi_Tratado_com_Larvi -> foi_tratado;
- opcao 'nao' da lista xv2ud66 renomeada n_o -> nao;
- tratamento ja vem fora do repetidor de tubitos (nivel do imovel).

liraa_xlsform.gerar e liraa_kobo._tratamento passam a usar os novos nomes,
mantendo leitura dos nomes legados. Sem migracao de banco. Versao 1.69.1.
47 testes LIRAa e regressao completa (807) aprovados.
</commit_message>
<xml_diff>
--- a/app_core/data/liraa_kobo_base.xlsx
+++ b/app_core/data/liraa_kobo_base.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="286">
   <si>
     <t>type</t>
   </si>
@@ -249,15 +249,15 @@
     <t>Digite em qual depósito foi coletada a amostra</t>
   </si>
   <si>
-    <t>group_rb5ho54</t>
+    <t>end_repeat</t>
+  </si>
+  <si>
+    <t>tratamento_001</t>
   </si>
   <si>
     <t>Tratamento</t>
   </si>
   <si>
-    <t>${Visita} = 'normal' or ${Visita} = 'recuperado'</t>
-  </si>
-  <si>
     <t>note</t>
   </si>
   <si>
@@ -270,7 +270,7 @@
     <t>select_one xv2ud66</t>
   </si>
   <si>
-    <t>O_im_vel_foi_Tratado_com_Larvi</t>
+    <t>foi_tratado</t>
   </si>
   <si>
     <t>O imóvel foi Tratado com Larvicida BTI?</t>
@@ -282,7 +282,7 @@
     <t>Quantidade carga (gr)</t>
   </si>
   <si>
-    <t>${O_im_vel_foi_Tratado_com_Larvi} = 'sim'</t>
+    <t>${foi_tratado} = 'sim'</t>
   </si>
   <si>
     <t>Quantidade_dep_sitos_tratados</t>
@@ -291,9 +291,6 @@
     <t>Quantidade depósitos tratados</t>
   </si>
   <si>
-    <t>end_repeat</t>
-  </si>
-  <si>
     <t>list_name</t>
   </si>
   <si>
@@ -870,7 +867,7 @@
     <t>Sim</t>
   </si>
   <si>
-    <t>n_o</t>
+    <t>nao</t>
   </si>
   <si>
     <t>Não</t>
@@ -1573,33 +1570,18 @@
     </row>
     <row r="22" spans="1:9">
       <c r="A22" t="s">
-        <v>30</v>
-      </c>
-      <c r="B22" t="s">
         <v>77</v>
-      </c>
-      <c r="C22" t="s">
-        <v>78</v>
-      </c>
-      <c r="F22" t="s">
-        <v>33</v>
-      </c>
-      <c r="I22" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="23" spans="1:9">
       <c r="A23" t="s">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C23" t="s">
-        <v>81</v>
-      </c>
-      <c r="D23" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F23" t="s">
         <v>33</v>
@@ -1607,47 +1589,47 @@
     </row>
     <row r="24" spans="1:9">
       <c r="A24" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B24" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C24" t="s">
-        <v>85</v>
+        <v>81</v>
+      </c>
+      <c r="D24" t="s">
+        <v>82</v>
       </c>
       <c r="F24" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" t="s">
-        <v>39</v>
+        <v>83</v>
       </c>
       <c r="B25" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C25" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F25" t="s">
-        <v>33</v>
-      </c>
-      <c r="I25" t="s">
-        <v>88</v>
+        <v>18</v>
       </c>
     </row>
     <row r="26" spans="1:9">
       <c r="A26" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C26" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F26" t="s">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="I26" t="s">
         <v>88</v>
@@ -1655,12 +1637,24 @@
     </row>
     <row r="27" spans="1:9">
       <c r="A27" t="s">
-        <v>64</v>
+        <v>52</v>
+      </c>
+      <c r="B27" t="s">
+        <v>89</v>
+      </c>
+      <c r="C27" t="s">
+        <v>90</v>
+      </c>
+      <c r="F27" t="s">
+        <v>18</v>
+      </c>
+      <c r="I27" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="28" spans="1:9">
       <c r="A28" t="s">
-        <v>91</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1675,7 +1669,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -1684,29 +1678,29 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" t="s">
         <v>94</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>95</v>
-      </c>
-      <c r="C2" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C3" t="s">
         <v>97</v>
-      </c>
-      <c r="C3" t="s">
-        <v>98</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -1714,13 +1708,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" t="s">
         <v>99</v>
-      </c>
-      <c r="C4" t="s">
-        <v>100</v>
       </c>
       <c r="D4">
         <v>2</v>
@@ -1728,13 +1722,13 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C5" t="s">
         <v>101</v>
-      </c>
-      <c r="C5" t="s">
-        <v>102</v>
       </c>
       <c r="D5">
         <v>3</v>
@@ -1742,13 +1736,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" t="s">
         <v>103</v>
-      </c>
-      <c r="C6" t="s">
-        <v>104</v>
       </c>
       <c r="D6">
         <v>4</v>
@@ -1756,13 +1750,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B7" t="s">
+        <v>104</v>
+      </c>
+      <c r="C7" t="s">
         <v>105</v>
-      </c>
-      <c r="C7" t="s">
-        <v>106</v>
       </c>
       <c r="D7">
         <v>5</v>
@@ -1770,13 +1764,13 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" t="s">
         <v>107</v>
-      </c>
-      <c r="C8" t="s">
-        <v>108</v>
       </c>
       <c r="D8">
         <v>6</v>
@@ -1784,13 +1778,13 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" t="s">
         <v>109</v>
-      </c>
-      <c r="C9" t="s">
-        <v>110</v>
       </c>
       <c r="D9">
         <v>7</v>
@@ -1798,13 +1792,13 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B10" t="s">
+        <v>110</v>
+      </c>
+      <c r="C10" t="s">
         <v>111</v>
-      </c>
-      <c r="C10" t="s">
-        <v>112</v>
       </c>
       <c r="D10">
         <v>8</v>
@@ -1812,13 +1806,13 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B11" t="s">
+        <v>112</v>
+      </c>
+      <c r="C11" t="s">
         <v>113</v>
-      </c>
-      <c r="C11" t="s">
-        <v>114</v>
       </c>
       <c r="D11">
         <v>9</v>
@@ -1826,13 +1820,13 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B12" t="s">
+        <v>114</v>
+      </c>
+      <c r="C12" t="s">
         <v>115</v>
-      </c>
-      <c r="C12" t="s">
-        <v>116</v>
       </c>
       <c r="D12">
         <v>10</v>
@@ -1840,13 +1834,13 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B13" t="s">
+        <v>116</v>
+      </c>
+      <c r="C13" t="s">
         <v>117</v>
-      </c>
-      <c r="C13" t="s">
-        <v>118</v>
       </c>
       <c r="D13">
         <v>11</v>
@@ -1854,13 +1848,13 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B14" t="s">
+        <v>118</v>
+      </c>
+      <c r="C14" t="s">
         <v>119</v>
-      </c>
-      <c r="C14" t="s">
-        <v>120</v>
       </c>
       <c r="D14">
         <v>12</v>
@@ -1868,13 +1862,13 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B15" t="s">
+        <v>120</v>
+      </c>
+      <c r="C15" t="s">
         <v>121</v>
-      </c>
-      <c r="C15" t="s">
-        <v>122</v>
       </c>
       <c r="D15">
         <v>13</v>
@@ -1882,13 +1876,13 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B16" t="s">
+        <v>122</v>
+      </c>
+      <c r="C16" t="s">
         <v>123</v>
-      </c>
-      <c r="C16" t="s">
-        <v>124</v>
       </c>
       <c r="D16">
         <v>14</v>
@@ -1896,13 +1890,13 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B17" t="s">
+        <v>124</v>
+      </c>
+      <c r="C17" t="s">
         <v>125</v>
-      </c>
-      <c r="C17" t="s">
-        <v>126</v>
       </c>
       <c r="D17">
         <v>15</v>
@@ -1910,13 +1904,13 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B18" t="s">
+        <v>126</v>
+      </c>
+      <c r="C18" t="s">
         <v>127</v>
-      </c>
-      <c r="C18" t="s">
-        <v>128</v>
       </c>
       <c r="D18">
         <v>17</v>
@@ -1924,13 +1918,13 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C19" t="s">
         <v>129</v>
-      </c>
-      <c r="C19" t="s">
-        <v>130</v>
       </c>
       <c r="D19">
         <v>19</v>
@@ -1938,13 +1932,13 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B20" t="s">
+        <v>130</v>
+      </c>
+      <c r="C20" t="s">
         <v>131</v>
-      </c>
-      <c r="C20" t="s">
-        <v>132</v>
       </c>
       <c r="D20">
         <v>20</v>
@@ -1952,35 +1946,35 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B21" t="s">
+        <v>132</v>
+      </c>
+      <c r="C21" t="s">
         <v>133</v>
-      </c>
-      <c r="C21" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" t="s">
+        <v>134</v>
+      </c>
+      <c r="B22" t="s">
         <v>135</v>
       </c>
-      <c r="B22" t="s">
-        <v>136</v>
-      </c>
       <c r="C22" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B23" t="s">
+        <v>136</v>
+      </c>
+      <c r="C23" t="s">
         <v>137</v>
-      </c>
-      <c r="C23" t="s">
-        <v>138</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -1988,13 +1982,13 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B24" t="s">
+        <v>138</v>
+      </c>
+      <c r="C24" t="s">
         <v>139</v>
-      </c>
-      <c r="C24" t="s">
-        <v>140</v>
       </c>
       <c r="D24">
         <v>2</v>
@@ -2002,13 +1996,13 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B25" t="s">
+        <v>140</v>
+      </c>
+      <c r="C25" t="s">
         <v>141</v>
-      </c>
-      <c r="C25" t="s">
-        <v>142</v>
       </c>
       <c r="D25">
         <v>3</v>
@@ -2016,13 +2010,13 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B26" t="s">
+        <v>142</v>
+      </c>
+      <c r="C26" t="s">
         <v>143</v>
-      </c>
-      <c r="C26" t="s">
-        <v>144</v>
       </c>
       <c r="D26">
         <v>4</v>
@@ -2030,13 +2024,13 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B27" t="s">
+        <v>144</v>
+      </c>
+      <c r="C27" t="s">
         <v>145</v>
-      </c>
-      <c r="C27" t="s">
-        <v>146</v>
       </c>
       <c r="D27">
         <v>5</v>
@@ -2044,13 +2038,13 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B28" t="s">
+        <v>146</v>
+      </c>
+      <c r="C28" t="s">
         <v>147</v>
-      </c>
-      <c r="C28" t="s">
-        <v>148</v>
       </c>
       <c r="D28">
         <v>6</v>
@@ -2058,13 +2052,13 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B29" t="s">
+        <v>148</v>
+      </c>
+      <c r="C29" t="s">
         <v>149</v>
-      </c>
-      <c r="C29" t="s">
-        <v>150</v>
       </c>
       <c r="D29">
         <v>7</v>
@@ -2072,13 +2066,13 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B30" t="s">
+        <v>150</v>
+      </c>
+      <c r="C30" t="s">
         <v>151</v>
-      </c>
-      <c r="C30" t="s">
-        <v>152</v>
       </c>
       <c r="D30">
         <v>8</v>
@@ -2086,13 +2080,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B31" t="s">
+        <v>152</v>
+      </c>
+      <c r="C31" t="s">
         <v>153</v>
-      </c>
-      <c r="C31" t="s">
-        <v>154</v>
       </c>
       <c r="D31">
         <v>9</v>
@@ -2100,13 +2094,13 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B32" t="s">
+        <v>154</v>
+      </c>
+      <c r="C32" t="s">
         <v>155</v>
-      </c>
-      <c r="C32" t="s">
-        <v>156</v>
       </c>
       <c r="D32">
         <v>10</v>
@@ -2114,13 +2108,13 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B33" t="s">
+        <v>156</v>
+      </c>
+      <c r="C33" t="s">
         <v>157</v>
-      </c>
-      <c r="C33" t="s">
-        <v>158</v>
       </c>
       <c r="D33">
         <v>11</v>
@@ -2128,13 +2122,13 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B34" t="s">
+        <v>158</v>
+      </c>
+      <c r="C34" t="s">
         <v>159</v>
-      </c>
-      <c r="C34" t="s">
-        <v>160</v>
       </c>
       <c r="D34">
         <v>12</v>
@@ -2142,13 +2136,13 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B35" t="s">
+        <v>160</v>
+      </c>
+      <c r="C35" t="s">
         <v>161</v>
-      </c>
-      <c r="C35" t="s">
-        <v>162</v>
       </c>
       <c r="D35">
         <v>13</v>
@@ -2156,13 +2150,13 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B36" t="s">
+        <v>162</v>
+      </c>
+      <c r="C36" t="s">
         <v>163</v>
-      </c>
-      <c r="C36" t="s">
-        <v>164</v>
       </c>
       <c r="D36">
         <v>14</v>
@@ -2170,13 +2164,13 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B37" t="s">
+        <v>164</v>
+      </c>
+      <c r="C37" t="s">
         <v>165</v>
-      </c>
-      <c r="C37" t="s">
-        <v>166</v>
       </c>
       <c r="D37">
         <v>15</v>
@@ -2184,13 +2178,13 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B38" t="s">
+        <v>166</v>
+      </c>
+      <c r="C38" t="s">
         <v>167</v>
-      </c>
-      <c r="C38" t="s">
-        <v>168</v>
       </c>
       <c r="D38">
         <v>16</v>
@@ -2198,13 +2192,13 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B39" t="s">
+        <v>168</v>
+      </c>
+      <c r="C39" t="s">
         <v>169</v>
-      </c>
-      <c r="C39" t="s">
-        <v>170</v>
       </c>
       <c r="D39">
         <v>17</v>
@@ -2212,13 +2206,13 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B40" t="s">
+        <v>170</v>
+      </c>
+      <c r="C40" t="s">
         <v>171</v>
-      </c>
-      <c r="C40" t="s">
-        <v>172</v>
       </c>
       <c r="D40">
         <v>18</v>
@@ -2226,13 +2220,13 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B41" t="s">
+        <v>172</v>
+      </c>
+      <c r="C41" t="s">
         <v>173</v>
-      </c>
-      <c r="C41" t="s">
-        <v>174</v>
       </c>
       <c r="D41">
         <v>19</v>
@@ -2240,13 +2234,13 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B42" t="s">
+        <v>174</v>
+      </c>
+      <c r="C42" t="s">
         <v>175</v>
-      </c>
-      <c r="C42" t="s">
-        <v>176</v>
       </c>
       <c r="D42">
         <v>20</v>
@@ -2254,13 +2248,13 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B43" t="s">
+        <v>176</v>
+      </c>
+      <c r="C43" t="s">
         <v>177</v>
-      </c>
-      <c r="C43" t="s">
-        <v>178</v>
       </c>
       <c r="D43">
         <v>21</v>
@@ -2268,13 +2262,13 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B44" t="s">
+        <v>178</v>
+      </c>
+      <c r="C44" t="s">
         <v>179</v>
-      </c>
-      <c r="C44" t="s">
-        <v>180</v>
       </c>
       <c r="D44">
         <v>22</v>
@@ -2282,13 +2276,13 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B45" t="s">
+        <v>180</v>
+      </c>
+      <c r="C45" t="s">
         <v>181</v>
-      </c>
-      <c r="C45" t="s">
-        <v>182</v>
       </c>
       <c r="D45">
         <v>23</v>
@@ -2296,13 +2290,13 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B46" t="s">
+        <v>182</v>
+      </c>
+      <c r="C46" t="s">
         <v>183</v>
-      </c>
-      <c r="C46" t="s">
-        <v>184</v>
       </c>
       <c r="D46">
         <v>24</v>
@@ -2310,13 +2304,13 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B47" t="s">
+        <v>184</v>
+      </c>
+      <c r="C47" t="s">
         <v>185</v>
-      </c>
-      <c r="C47" t="s">
-        <v>186</v>
       </c>
       <c r="D47">
         <v>25</v>
@@ -2324,13 +2318,13 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B48" t="s">
+        <v>186</v>
+      </c>
+      <c r="C48" t="s">
         <v>187</v>
-      </c>
-      <c r="C48" t="s">
-        <v>188</v>
       </c>
       <c r="D48">
         <v>26</v>
@@ -2338,13 +2332,13 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B49" t="s">
+        <v>188</v>
+      </c>
+      <c r="C49" t="s">
         <v>189</v>
-      </c>
-      <c r="C49" t="s">
-        <v>190</v>
       </c>
       <c r="D49">
         <v>27</v>
@@ -2352,13 +2346,13 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B50" t="s">
+        <v>190</v>
+      </c>
+      <c r="C50" t="s">
         <v>191</v>
-      </c>
-      <c r="C50" t="s">
-        <v>192</v>
       </c>
       <c r="D50">
         <v>28</v>
@@ -2366,13 +2360,13 @@
     </row>
     <row r="51" spans="1:4">
       <c r="A51" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B51" t="s">
+        <v>192</v>
+      </c>
+      <c r="C51" t="s">
         <v>193</v>
-      </c>
-      <c r="C51" t="s">
-        <v>194</v>
       </c>
       <c r="D51">
         <v>29</v>
@@ -2380,13 +2374,13 @@
     </row>
     <row r="52" spans="1:4">
       <c r="A52" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B52" t="s">
+        <v>194</v>
+      </c>
+      <c r="C52" t="s">
         <v>195</v>
-      </c>
-      <c r="C52" t="s">
-        <v>196</v>
       </c>
       <c r="D52">
         <v>30</v>
@@ -2394,13 +2388,13 @@
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B53" t="s">
+        <v>196</v>
+      </c>
+      <c r="C53" t="s">
         <v>197</v>
-      </c>
-      <c r="C53" t="s">
-        <v>198</v>
       </c>
       <c r="D53">
         <v>31</v>
@@ -2408,13 +2402,13 @@
     </row>
     <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B54" t="s">
+        <v>198</v>
+      </c>
+      <c r="C54" t="s">
         <v>199</v>
-      </c>
-      <c r="C54" t="s">
-        <v>200</v>
       </c>
       <c r="D54">
         <v>32</v>
@@ -2422,13 +2416,13 @@
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B55" t="s">
+        <v>200</v>
+      </c>
+      <c r="C55" t="s">
         <v>201</v>
-      </c>
-      <c r="C55" t="s">
-        <v>202</v>
       </c>
       <c r="D55">
         <v>33</v>
@@ -2436,13 +2430,13 @@
     </row>
     <row r="56" spans="1:4">
       <c r="A56" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B56" t="s">
+        <v>202</v>
+      </c>
+      <c r="C56" t="s">
         <v>203</v>
-      </c>
-      <c r="C56" t="s">
-        <v>204</v>
       </c>
       <c r="D56">
         <v>34</v>
@@ -2450,13 +2444,13 @@
     </row>
     <row r="57" spans="1:4">
       <c r="A57" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B57" t="s">
+        <v>204</v>
+      </c>
+      <c r="C57" t="s">
         <v>205</v>
-      </c>
-      <c r="C57" t="s">
-        <v>206</v>
       </c>
       <c r="D57">
         <v>35</v>
@@ -2464,13 +2458,13 @@
     </row>
     <row r="58" spans="1:4">
       <c r="A58" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B58" t="s">
+        <v>206</v>
+      </c>
+      <c r="C58" t="s">
         <v>207</v>
-      </c>
-      <c r="C58" t="s">
-        <v>208</v>
       </c>
       <c r="D58">
         <v>36</v>
@@ -2478,13 +2472,13 @@
     </row>
     <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B59" t="s">
+        <v>208</v>
+      </c>
+      <c r="C59" t="s">
         <v>209</v>
-      </c>
-      <c r="C59" t="s">
-        <v>210</v>
       </c>
       <c r="D59">
         <v>37</v>
@@ -2492,13 +2486,13 @@
     </row>
     <row r="60" spans="1:4">
       <c r="A60" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B60" t="s">
+        <v>210</v>
+      </c>
+      <c r="C60" t="s">
         <v>211</v>
-      </c>
-      <c r="C60" t="s">
-        <v>212</v>
       </c>
       <c r="D60">
         <v>38</v>
@@ -2506,13 +2500,13 @@
     </row>
     <row r="61" spans="1:4">
       <c r="A61" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B61" t="s">
+        <v>212</v>
+      </c>
+      <c r="C61" t="s">
         <v>213</v>
-      </c>
-      <c r="C61" t="s">
-        <v>214</v>
       </c>
       <c r="D61">
         <v>39</v>
@@ -2520,13 +2514,13 @@
     </row>
     <row r="62" spans="1:4">
       <c r="A62" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B62" t="s">
+        <v>214</v>
+      </c>
+      <c r="C62" t="s">
         <v>215</v>
-      </c>
-      <c r="C62" t="s">
-        <v>216</v>
       </c>
       <c r="D62">
         <v>40</v>
@@ -2534,13 +2528,13 @@
     </row>
     <row r="63" spans="1:4">
       <c r="A63" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B63" t="s">
+        <v>216</v>
+      </c>
+      <c r="C63" t="s">
         <v>217</v>
-      </c>
-      <c r="C63" t="s">
-        <v>218</v>
       </c>
       <c r="D63">
         <v>41</v>
@@ -2548,13 +2542,13 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B64" t="s">
+        <v>218</v>
+      </c>
+      <c r="C64" t="s">
         <v>219</v>
-      </c>
-      <c r="C64" t="s">
-        <v>220</v>
       </c>
       <c r="D64">
         <v>42</v>
@@ -2562,13 +2556,13 @@
     </row>
     <row r="65" spans="1:4">
       <c r="A65" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B65" t="s">
+        <v>220</v>
+      </c>
+      <c r="C65" t="s">
         <v>221</v>
-      </c>
-      <c r="C65" t="s">
-        <v>222</v>
       </c>
       <c r="D65">
         <v>43</v>
@@ -2576,13 +2570,13 @@
     </row>
     <row r="66" spans="1:4">
       <c r="A66" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B66" t="s">
+        <v>222</v>
+      </c>
+      <c r="C66" t="s">
         <v>223</v>
-      </c>
-      <c r="C66" t="s">
-        <v>224</v>
       </c>
       <c r="D66">
         <v>44</v>
@@ -2590,13 +2584,13 @@
     </row>
     <row r="67" spans="1:4">
       <c r="A67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B67" t="s">
+        <v>224</v>
+      </c>
+      <c r="C67" t="s">
         <v>225</v>
-      </c>
-      <c r="C67" t="s">
-        <v>226</v>
       </c>
       <c r="D67">
         <v>45</v>
@@ -2604,13 +2598,13 @@
     </row>
     <row r="68" spans="1:4">
       <c r="A68" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B68" t="s">
+        <v>226</v>
+      </c>
+      <c r="C68" t="s">
         <v>227</v>
-      </c>
-      <c r="C68" t="s">
-        <v>228</v>
       </c>
       <c r="D68">
         <v>46</v>
@@ -2618,13 +2612,13 @@
     </row>
     <row r="69" spans="1:4">
       <c r="A69" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B69" t="s">
+        <v>228</v>
+      </c>
+      <c r="C69" t="s">
         <v>229</v>
-      </c>
-      <c r="C69" t="s">
-        <v>230</v>
       </c>
       <c r="D69">
         <v>47</v>
@@ -2632,13 +2626,13 @@
     </row>
     <row r="70" spans="1:4">
       <c r="A70" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B70" t="s">
+        <v>230</v>
+      </c>
+      <c r="C70" t="s">
         <v>231</v>
-      </c>
-      <c r="C70" t="s">
-        <v>232</v>
       </c>
       <c r="D70">
         <v>48</v>
@@ -2646,13 +2640,13 @@
     </row>
     <row r="71" spans="1:4">
       <c r="A71" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B71" t="s">
+        <v>232</v>
+      </c>
+      <c r="C71" t="s">
         <v>233</v>
-      </c>
-      <c r="C71" t="s">
-        <v>234</v>
       </c>
       <c r="D71">
         <v>49</v>
@@ -2660,13 +2654,13 @@
     </row>
     <row r="72" spans="1:4">
       <c r="A72" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B72" t="s">
+        <v>234</v>
+      </c>
+      <c r="C72" t="s">
         <v>235</v>
-      </c>
-      <c r="C72" t="s">
-        <v>236</v>
       </c>
       <c r="D72">
         <v>50</v>
@@ -2674,13 +2668,13 @@
     </row>
     <row r="73" spans="1:4">
       <c r="A73" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B73" t="s">
+        <v>236</v>
+      </c>
+      <c r="C73" t="s">
         <v>237</v>
-      </c>
-      <c r="C73" t="s">
-        <v>238</v>
       </c>
       <c r="D73">
         <v>51</v>
@@ -2688,13 +2682,13 @@
     </row>
     <row r="74" spans="1:4">
       <c r="A74" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B74" t="s">
+        <v>238</v>
+      </c>
+      <c r="C74" t="s">
         <v>239</v>
-      </c>
-      <c r="C74" t="s">
-        <v>240</v>
       </c>
       <c r="D74">
         <v>52</v>
@@ -2702,13 +2696,13 @@
     </row>
     <row r="75" spans="1:4">
       <c r="A75" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B75" t="s">
+        <v>240</v>
+      </c>
+      <c r="C75" t="s">
         <v>241</v>
-      </c>
-      <c r="C75" t="s">
-        <v>242</v>
       </c>
       <c r="D75">
         <v>53</v>
@@ -2716,13 +2710,13 @@
     </row>
     <row r="76" spans="1:4">
       <c r="A76" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B76" t="s">
+        <v>242</v>
+      </c>
+      <c r="C76" t="s">
         <v>243</v>
-      </c>
-      <c r="C76" t="s">
-        <v>244</v>
       </c>
       <c r="D76">
         <v>54</v>
@@ -2730,13 +2724,13 @@
     </row>
     <row r="77" spans="1:4">
       <c r="A77" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B77" t="s">
+        <v>244</v>
+      </c>
+      <c r="C77" t="s">
         <v>245</v>
-      </c>
-      <c r="C77" t="s">
-        <v>246</v>
       </c>
       <c r="D77">
         <v>55</v>
@@ -2744,24 +2738,24 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" t="s">
+        <v>246</v>
+      </c>
+      <c r="B78" t="s">
         <v>247</v>
       </c>
-      <c r="B78" t="s">
+      <c r="C78" t="s">
         <v>248</v>
-      </c>
-      <c r="C78" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="79" spans="1:4">
       <c r="A79" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B79" t="s">
+        <v>249</v>
+      </c>
+      <c r="C79" t="s">
         <v>250</v>
-      </c>
-      <c r="C79" t="s">
-        <v>251</v>
       </c>
       <c r="D79">
         <v>2</v>
@@ -2769,13 +2763,13 @@
     </row>
     <row r="80" spans="1:4">
       <c r="A80" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B80" t="s">
+        <v>251</v>
+      </c>
+      <c r="C80" t="s">
         <v>252</v>
-      </c>
-      <c r="C80" t="s">
-        <v>253</v>
       </c>
       <c r="D80">
         <v>3</v>
@@ -2783,13 +2777,13 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B81" t="s">
+        <v>253</v>
+      </c>
+      <c r="C81" t="s">
         <v>254</v>
-      </c>
-      <c r="C81" t="s">
-        <v>255</v>
       </c>
       <c r="D81">
         <v>4</v>
@@ -2797,13 +2791,13 @@
     </row>
     <row r="82" spans="1:4">
       <c r="A82" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B82" t="s">
+        <v>255</v>
+      </c>
+      <c r="C82" t="s">
         <v>256</v>
-      </c>
-      <c r="C82" t="s">
-        <v>257</v>
       </c>
       <c r="D82">
         <v>5</v>
@@ -2811,13 +2805,13 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B83" t="s">
+        <v>257</v>
+      </c>
+      <c r="C83" t="s">
         <v>258</v>
-      </c>
-      <c r="C83" t="s">
-        <v>259</v>
       </c>
       <c r="D83">
         <v>6</v>
@@ -2825,13 +2819,13 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B84" t="s">
+        <v>259</v>
+      </c>
+      <c r="C84" t="s">
         <v>260</v>
-      </c>
-      <c r="C84" t="s">
-        <v>261</v>
       </c>
       <c r="D84">
         <v>7</v>
@@ -2839,13 +2833,13 @@
     </row>
     <row r="85" spans="1:4">
       <c r="A85" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B85" t="s">
+        <v>261</v>
+      </c>
+      <c r="C85" t="s">
         <v>262</v>
-      </c>
-      <c r="C85" t="s">
-        <v>263</v>
       </c>
       <c r="D85">
         <v>8</v>
@@ -2853,13 +2847,13 @@
     </row>
     <row r="86" spans="1:4">
       <c r="A86" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B86" t="s">
+        <v>263</v>
+      </c>
+      <c r="C86" t="s">
         <v>264</v>
-      </c>
-      <c r="C86" t="s">
-        <v>265</v>
       </c>
       <c r="D86">
         <v>9</v>
@@ -2867,13 +2861,13 @@
     </row>
     <row r="87" spans="1:4">
       <c r="A87" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B87" t="s">
+        <v>265</v>
+      </c>
+      <c r="C87" t="s">
         <v>266</v>
-      </c>
-      <c r="C87" t="s">
-        <v>267</v>
       </c>
       <c r="D87">
         <v>10</v>
@@ -2881,13 +2875,13 @@
     </row>
     <row r="88" spans="1:4">
       <c r="A88" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B88" t="s">
+        <v>267</v>
+      </c>
+      <c r="C88" t="s">
         <v>268</v>
-      </c>
-      <c r="C88" t="s">
-        <v>269</v>
       </c>
       <c r="D88">
         <v>11</v>
@@ -2895,13 +2889,13 @@
     </row>
     <row r="89" spans="1:4">
       <c r="A89" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B89" t="s">
+        <v>269</v>
+      </c>
+      <c r="C89" t="s">
         <v>270</v>
-      </c>
-      <c r="C89" t="s">
-        <v>271</v>
       </c>
       <c r="D89">
         <v>12</v>
@@ -2909,13 +2903,13 @@
     </row>
     <row r="90" spans="1:4">
       <c r="A90" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B90" t="s">
+        <v>271</v>
+      </c>
+      <c r="C90" t="s">
         <v>272</v>
-      </c>
-      <c r="C90" t="s">
-        <v>273</v>
       </c>
       <c r="D90">
         <v>13</v>
@@ -2923,13 +2917,13 @@
     </row>
     <row r="91" spans="1:4">
       <c r="A91" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B91" t="s">
+        <v>273</v>
+      </c>
+      <c r="C91" t="s">
         <v>274</v>
-      </c>
-      <c r="C91" t="s">
-        <v>275</v>
       </c>
       <c r="D91">
         <v>14</v>
@@ -2937,46 +2931,46 @@
     </row>
     <row r="92" spans="1:4">
       <c r="A92" t="s">
+        <v>275</v>
+      </c>
+      <c r="B92" t="s">
         <v>276</v>
       </c>
-      <c r="B92" t="s">
+      <c r="C92" t="s">
         <v>277</v>
-      </c>
-      <c r="C92" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="93" spans="1:4">
       <c r="A93" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B93" t="s">
+        <v>278</v>
+      </c>
+      <c r="C93" t="s">
         <v>279</v>
-      </c>
-      <c r="C93" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="94" spans="1:4">
       <c r="A94" t="s">
+        <v>280</v>
+      </c>
+      <c r="B94" t="s">
         <v>281</v>
       </c>
-      <c r="B94" t="s">
+      <c r="C94" t="s">
         <v>282</v>
-      </c>
-      <c r="C94" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="95" spans="1:4">
       <c r="A95" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B95" t="s">
+        <v>283</v>
+      </c>
+      <c r="C95" t="s">
         <v>284</v>
-      </c>
-      <c r="C95" t="s">
-        <v>285</v>
       </c>
     </row>
   </sheetData>
@@ -2991,7 +2985,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>